<commit_message>
Diagnostic to get the issues
</commit_message>
<xml_diff>
--- a/Visiting_Card_Data_ULTIMATE.xlsx
+++ b/Visiting_Card_Data_ULTIMATE.xlsx
@@ -440,9 +440,9 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="49" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -539,17 +539,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>URBANEDGE INFRA SOLUTIONS LLP</t>
+          <t>UR BA NED GE 50LUTTONS LLP</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>in | 8th Floor SkyTower Complex | Sure 395007</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ARCHITECT &amp; FOUND ER</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -558,10 +558,10 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="K2" t="n">
-        <v>0.77</v>
+        <v>0.89</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>

</xml_diff>